<commit_message>
Log weight through 2026-10-26 (79.1 kg), refit spline and plot
measure_weight skill; the workbook also carries the entries since the last
commit (2026-07-26).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/martysweight.xlsx
+++ b/inst/extdata/martysweight.xlsx
@@ -45852,6 +45852,237 @@
       </c>
       <c r="G2419"/>
     </row>
+    <row r="2420">
+      <c r="A2420" s="1" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B2420" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2420" t="n">
+        <v>32</v>
+      </c>
+      <c r="D2420" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2420" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2420" t="n">
+        <v>77.9</v>
+      </c>
+      <c r="G2420"/>
+    </row>
+    <row r="2421">
+      <c r="A2421" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B2421" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2421" t="n">
+        <v>4</v>
+      </c>
+      <c r="D2421" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2421" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2421" t="n">
+        <v>78.2</v>
+      </c>
+      <c r="G2421"/>
+    </row>
+    <row r="2422">
+      <c r="A2422" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B2422" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2422" t="n">
+        <v>22</v>
+      </c>
+      <c r="D2422" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2422" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2422" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="G2422"/>
+    </row>
+    <row r="2423">
+      <c r="A2423" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B2423" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2423" t="n">
+        <v>49</v>
+      </c>
+      <c r="D2423" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2423" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2423" t="n">
+        <v>77.7</v>
+      </c>
+      <c r="G2423"/>
+    </row>
+    <row r="2424">
+      <c r="A2424" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B2424" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2424" t="n">
+        <v>7</v>
+      </c>
+      <c r="D2424" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2424" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2424" t="n">
+        <v>77.9</v>
+      </c>
+      <c r="G2424"/>
+    </row>
+    <row r="2425">
+      <c r="A2425" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B2425" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2425" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2425" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2425" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2425" t="n">
+        <v>78.2</v>
+      </c>
+      <c r="G2425"/>
+    </row>
+    <row r="2426">
+      <c r="A2426" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B2426" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2426" t="n">
+        <v>20</v>
+      </c>
+      <c r="D2426" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2426" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2426" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="G2426"/>
+    </row>
+    <row r="2427">
+      <c r="A2427" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B2427" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2427" t="n">
+        <v>11</v>
+      </c>
+      <c r="D2427" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2427" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2427" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="G2427"/>
+    </row>
+    <row r="2428">
+      <c r="A2428" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B2428" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2428" t="n">
+        <v>55</v>
+      </c>
+      <c r="D2428" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2428" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2428" t="n">
+        <v>77.9</v>
+      </c>
+      <c r="G2428"/>
+    </row>
+    <row r="2429">
+      <c r="A2429" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B2429" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2429" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2429" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2429" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2429" t="n">
+        <v>78.5</v>
+      </c>
+      <c r="G2429"/>
+    </row>
+    <row r="2430">
+      <c r="A2430" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B2430" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2430" t="n">
+        <v>57</v>
+      </c>
+      <c r="D2430" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2430" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2430" t="n">
+        <v>79.1</v>
+      </c>
+      <c r="G2430"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>